<commit_message>
fixed size_max pipeline_large and set capex to 0 in piecewise formualtion of CaL and oxy
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/CementHybridCCS_data/cement_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\CementHybridCCS_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0064542-306E-4AE4-8E2A-76DCB265744D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63AFDCFD-5607-44CC-996A-D0FCDE1AB878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C0ECAA26-0769-408D-9398-31AECF4E3649}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_oxyfuel" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{1034DA71-6109-44C0-9094-3BCE06243C3C}">
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{1034DA71-6109-44C0-9094-3BCE06243C3C}">
       <text>
         <r>
           <rPr>
@@ -106,7 +106,7 @@
     <author>Bertoni, L. (Luca)</author>
   </authors>
   <commentList>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{59747281-07D3-4DCE-BDD0-69E2E6DC2FBF}">
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{59747281-07D3-4DCE-BDD0-69E2E6DC2FBF}">
       <text>
         <r>
           <rPr>
@@ -1175,14 +1175,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D08EB36-8885-41F7-B3E9-60083815A79B}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1190,28 +1190,36 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>75</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <v>50760000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>125</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>72350000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="21">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="21">
         <v>220</v>
       </c>
-      <c r="B4" s="21">
-        <f>_xlfn.FORECAST.LINEAR($A$4, B2:B3, $A$2:$A$3)</f>
+      <c r="B5" s="21">
+        <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
         <v>113371000</v>
       </c>
     </row>
@@ -1223,14 +1231,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447E0F8A-1C59-405C-B3D0-EB533A2330E6}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1238,46 +1246,54 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
         <f>calculations!D19</f>
         <v>4.4302472880300003</v>
       </c>
-      <c r="B2">
+      <c r="B3">
         <f>calculations!D20</f>
         <v>13962331.812465826</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
         <f>calculations!G19</f>
         <v>14.767490960100002</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <f>calculations!G20</f>
         <v>25360000.000000007</v>
       </c>
-      <c r="C3">
-        <f>B3/A3</f>
+      <c r="C4">
+        <f>B4/A4</f>
         <v>1717285.6288532494</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
         <f>calculations!G6</f>
         <v>24.418823252400006</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <f>calculations!G7</f>
         <v>26820000.000000007</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="21">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="21">
         <v>50</v>
       </c>
-      <c r="B5" s="21">
-        <f>_xlfn.FORECAST.LINEAR($A$5, B3:B4, $A$3:$A$4)</f>
+      <c r="B6" s="21">
+        <f>_xlfn.FORECAST.LINEAR($A$6, B4:B5, $A$4:$A$5)</f>
         <v>30689778.48449932</v>
       </c>
     </row>
@@ -1291,9 +1307,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E17DFFB0-96B6-4F96-B3DF-E2D36B37C43F}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1307,7 +1323,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1321,7 +1337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>75</v>
       </c>
@@ -1335,7 +1351,7 @@
         <v>61000000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>125</v>
       </c>
@@ -1349,7 +1365,7 @@
         <v>71600000</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="21">
         <v>220</v>
       </c>
@@ -1375,15 +1391,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8995DE27-F5E7-40F1-8502-5CC793EB5921}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1397,7 +1413,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -1411,7 +1427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>calculations!D19</f>
         <v>4.4302472880300003</v>
@@ -1428,7 +1444,7 @@
         <v>10684945.673991</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <f>calculations!G19</f>
         <v>14.767490960100002</v>
@@ -1446,7 +1462,7 @@
         <v>16588739.769484399</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <f>calculations!G6</f>
         <v>24.418823252400006</v>
@@ -1464,7 +1480,7 @@
         <v>19939806.622189701</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="21">
         <v>50</v>
       </c>
@@ -1490,17 +1506,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69712579-C7D8-42EE-9801-1FD637D0A17F}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -1509,7 +1525,7 @@
         <v>0.3128088466592428</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -1518,7 +1534,7 @@
         <v>7.833563329433206E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -1527,7 +1543,7 @@
         <v>3.8587338925408297E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -1544,12 +1560,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21185F42-04E5-4941-B133-36036095D1EF}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>53</v>
       </c>
@@ -1563,7 +1579,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -1577,7 +1593,7 @@
         <v>0.13739152500000001</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1591,10 +1607,10 @@
         <v>8.9737128657946114E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" s="20"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D7" s="20"/>
     </row>
   </sheetData>
@@ -1605,16 +1621,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB78D47C-565F-4352-814A-A37F11C35FBF}">
   <dimension ref="A1:T57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.88671875" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="52" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="16.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" ht="18.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22" t="s">
         <v>3</v>
       </c>
@@ -1634,7 +1650,7 @@
       <c r="S1" s="10"/>
       <c r="T1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="25" t="s">
         <v>4</v>
       </c>
@@ -1666,7 +1682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="27"/>
       <c r="B3" s="28"/>
       <c r="C3" s="1" t="s">
@@ -1706,7 +1722,7 @@
         <v>2999.91944736</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="27"/>
       <c r="B4" s="28"/>
       <c r="C4" s="33">
@@ -1746,7 +1762,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="29"/>
       <c r="B5" s="30"/>
       <c r="C5" s="33"/>
@@ -1780,7 +1796,7 @@
         <v>32.665832100000003</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
@@ -1825,7 +1841,7 @@
         <v>0.343073721</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>14</v>
       </c>
@@ -1868,7 +1884,7 @@
         <v>6.7830064590000019</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
@@ -1911,7 +1927,7 @@
         <v>32.322758379</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>16</v>
       </c>
@@ -1953,7 +1969,7 @@
         <v>29.496494612333333</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B10" s="16" t="s">
         <v>59</v>
       </c>
@@ -1998,7 +2014,7 @@
         <v>26.670230845666659</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B11" s="16" t="s">
         <v>60</v>
       </c>
@@ -2044,7 +2060,7 @@
         <v>0.98850272506734771</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B12" s="16" t="s">
         <v>61</v>
       </c>
@@ -2090,7 +2106,7 @@
         <v>5.1419803699999997</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="N13" s="3" t="s">
         <v>28</v>
       </c>
@@ -2113,7 +2129,7 @@
         <v>8.4990979400000004</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
@@ -2145,7 +2161,7 @@
         <v>24.018188706552724</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="25" t="s">
         <v>4</v>
       </c>
@@ -2179,7 +2195,7 @@
         <v>3.5409355499999999</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="27"/>
       <c r="B16" s="28"/>
       <c r="C16" s="1" t="s">
@@ -2219,7 +2235,7 @@
         <v>7.0372530900000001</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="27"/>
       <c r="B17" s="28"/>
       <c r="C17" s="33">
@@ -2259,7 +2275,7 @@
         <v>0.16516841700000001</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="29"/>
       <c r="B18" s="30"/>
       <c r="C18" s="33"/>
@@ -2289,7 +2305,7 @@
         <v>38.587338925408297</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="7" t="s">
         <v>13</v>
@@ -2335,7 +2351,7 @@
         <v>0.9422574090000001</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>14</v>
       </c>
@@ -2378,7 +2394,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B21" s="7" t="s">
         <v>15</v>
       </c>
@@ -2421,7 +2437,7 @@
         <v>34915.217199999999</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>16</v>
       </c>
@@ -2463,7 +2479,7 @@
         <v>-10.897028493447277</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B23" s="16" t="s">
         <v>59</v>
       </c>
@@ -2502,7 +2518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B24" s="16" t="s">
         <v>60</v>
       </c>
@@ -2548,7 +2564,7 @@
         <v>0.87964504737233462</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B25" s="16" t="s">
         <v>61</v>
       </c>
@@ -2594,7 +2610,7 @@
         <v>7203.3637644090004</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N26" s="3" t="s">
         <v>42</v>
       </c>
@@ -2617,7 +2633,7 @@
         <v>61.904815039006735</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N27" s="3" t="s">
         <v>38</v>
       </c>
@@ -2640,7 +2656,7 @@
         <v>9.8807884726655857</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="9"/>
@@ -2666,7 +2682,7 @@
         <v>4020.725250921625</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="4"/>
       <c r="C29" s="9"/>
@@ -2678,7 +2694,7 @@
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
     </row>
-    <row r="30" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="9"/>
@@ -2692,7 +2708,7 @@
       <c r="S30" s="10"/>
       <c r="T30" s="10"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="6"/>
@@ -2716,7 +2732,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -2742,7 +2758,7 @@
         <v>1799.9672083200001</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
@@ -2768,7 +2784,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -2794,7 +2810,7 @@
         <v>19.661164899999999</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
@@ -2820,7 +2836,7 @@
         <v>0.207687817</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -2846,7 +2862,7 @@
         <v>4.1020808222500005</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N37" s="3" t="s">
         <v>23</v>
       </c>
@@ -2869,7 +2885,7 @@
         <v>19.453477082999999</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>62</v>
       </c>
@@ -2902,7 +2918,7 @@
         <v>17.713778155222222</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>44</v>
       </c>
@@ -2935,7 +2951,7 @@
         <v>15.974079227444445</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>45</v>
       </c>
@@ -2968,7 +2984,7 @@
         <v>0.98841122610606125</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>46</v>
       </c>
@@ -3001,7 +3017,7 @@
         <v>3.1058323420000002</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N42" s="3" t="s">
         <v>28</v>
       </c>
@@ -3024,7 +3040,7 @@
         <v>5.1170056500000003</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N43" s="3" t="s">
         <v>29</v>
       </c>
@@ -3047,7 +3063,7 @@
         <v>14.592057884886959</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N44" s="3" t="s">
         <v>30</v>
       </c>
@@ -3070,7 +3086,7 @@
         <v>3.5572331500000001</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N45" s="3" t="s">
         <v>31</v>
       </c>
@@ -3093,7 +3109,7 @@
         <v>4.2368806800000005</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N46" s="3" t="s">
         <v>32</v>
       </c>
@@ -3116,7 +3132,7 @@
         <v>9.9445346300000001E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N47" s="3" t="s">
         <v>33</v>
       </c>
@@ -3139,7 +3155,7 @@
         <v>38.574472030429632</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N48" s="3" t="s">
         <v>34</v>
       </c>
@@ -3162,7 +3178,7 @@
         <v>0.56964816699999998</v>
       </c>
     </row>
-    <row r="49" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N49" s="15" t="s">
         <v>58</v>
       </c>
@@ -3185,7 +3201,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N50" s="3" t="s">
         <v>35</v>
       </c>
@@ -3208,7 +3224,7 @@
         <v>21030.427199999998</v>
       </c>
     </row>
-    <row r="51" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N51" s="3" t="s">
         <v>36</v>
       </c>
@@ -3231,7 +3247,7 @@
         <v>-6.4383693151130394</v>
       </c>
     </row>
-    <row r="52" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N52" s="3"/>
       <c r="O52" s="11"/>
       <c r="P52" s="11"/>
@@ -3248,7 +3264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N53" s="3" t="s">
         <v>41</v>
       </c>
@@ -3271,7 +3287,7 @@
         <v>0.89878949162663713</v>
       </c>
     </row>
-    <row r="54" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N54" s="3" t="s">
         <v>37</v>
       </c>
@@ -3294,7 +3310,7 @@
         <v>4336.8956744670004</v>
       </c>
     </row>
-    <row r="55" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N55" s="3" t="s">
         <v>42</v>
       </c>
@@ -3317,7 +3333,7 @@
         <v>61.926885243577217</v>
       </c>
     </row>
-    <row r="56" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="56" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N56" s="3" t="s">
         <v>38</v>
       </c>
@@ -3340,7 +3356,7 @@
         <v>9.9691968308401844</v>
       </c>
     </row>
-    <row r="57" spans="14:20" x14ac:dyDescent="0.3">
+    <row r="57" spans="14:20" x14ac:dyDescent="0.25">
       <c r="N57" s="3" t="s">
         <v>39</v>
       </c>
@@ -3365,6 +3381,14 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A15:B18"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:B5"/>
     <mergeCell ref="C2:G2"/>
@@ -3373,14 +3397,6 @@
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A15:B18"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>